<commit_message>
Migrate Screenshot Intelligence to Repository Platform
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B234"/>
+  <dimension ref="A1:B335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,2796 +431,4004 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Alert Management in Freshservice - An Overview</t>
+          <t>Operators | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002885-alert-management-in-freshservice-an-overview</t>
+          <t>https://help.savantlabs.io/en/articles/6245717-operators</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Set up alert management in Freshservice</t>
+          <t>AWS Athena Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003698-set-up-alert-management-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/6245797-aws-athena-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Automatically create alert-based incidents using Alert Rules</t>
+          <t>Amazon Redshift Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002729-automatically-create-alert-based-incidents-using-alert-rules</t>
+          <t>https://help.savantlabs.io/en/articles/6245801-amazon-redshift-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Working with alerts in Freshservice Alert Management</t>
+          <t>Google Drive Connection Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003697-working-with-alerts-in-freshservice-alert-management</t>
+          <t>https://help.savantlabs.io/en/articles/6245806-google-drive-connection-setup</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Learn all about Automated Grouping in Freshservice</t>
+          <t>Google Sheets Connection Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003799-learn-all-about-automated-grouping-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/6245809-google-sheets-connection-setup</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Integrate SolarWinds NPM with Freshservice Alert Management</t>
+          <t>Hubspot Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002747-integrate-solarwinds-npm-with-freshservice-alert-management</t>
+          <t>https://help.savantlabs.io/en/articles/6245810-hubspot-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Integrate New Relic APM with Freshservice Alert Management</t>
+          <t>MariaDB Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002803-integrate-new-relic-apm-with-freshservice-alert-management</t>
+          <t>https://help.savantlabs.io/en/articles/6245819-mariadb-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Integrate New Relic Synthetics with Freshservice Alert Management</t>
+          <t>Slack Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002838-integrate-new-relic-synthetics-with-freshservice-alert-management</t>
+          <t>https://help.savantlabs.io/en/articles/6245821-slack-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Integrate Pingdom with Freshservice Alert Management</t>
+          <t>Snowflake Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002839-integrate-pingdom-with-freshservice-alert-management</t>
+          <t>https://help.savantlabs.io/en/articles/6245824-snowflake-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Integrate Site 24x7 with Freshservice Alert Management</t>
+          <t>SSH Tunnel Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002876-integrate-site-24x7-with-freshservice-alert-management</t>
+          <t>https://help.savantlabs.io/en/articles/6245827-ssh-tunnel-setup</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Introducing Orchestration Center</t>
+          <t>Sales Lead-to-Account Analytics | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002961-introducing-orchestration-center</t>
+          <t>https://help.savantlabs.io/en/articles/6271020-sales-lead-to-account-analytics</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Orchestration FAQs</t>
+          <t>Pendo Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003144-orchestration-faqs</t>
+          <t>https://help.savantlabs.io/en/articles/6313955-pendo-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Workflow Execution Logs</t>
+          <t>Zendesk Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000011551-workflow-execution-logs</t>
+          <t>https://help.savantlabs.io/en/articles/6319201-zendesk-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Setting up the Orchestration Server</t>
+          <t>Greenhouse Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003259-setting-up-the-orchestration-server</t>
+          <t>https://help.savantlabs.io/en/articles/6319607-greenhouse-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>How to Reset the Secret Key of an Orchestration Server</t>
+          <t>Shopify Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003260-how-to-reset-the-secret-key-of-an-orchestration-server</t>
+          <t>https://help.savantlabs.io/en/articles/6322706-shopify-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Uninstalling the Orchestration Server</t>
+          <t>Salesforce Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003261-uninstalling-the-orchestration-server</t>
+          <t>https://help.savantlabs.io/en/articles/6322755-salesforce-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Troubleshooting Guide for Orchestration Server Issues</t>
+          <t>Dropbox Connection Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003393-troubleshooting-guide-for-orchestration-server-issues</t>
+          <t>https://help.savantlabs.io/en/articles/6322911-dropbox-connection-setup</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MS AD/Powershell/OSR - FAQ/L2s</t>
+          <t>AWS S3 Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004234-ms-ad-powershell-osr-faq-l2s</t>
+          <t>https://help.savantlabs.io/en/articles/6398804-aws-s3-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Learn all about Freshservice On-Call Management</t>
+          <t>MySQL Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003777-learn-all-about-freshservice-on-call-management</t>
+          <t>https://help.savantlabs.io/en/articles/6558726-mysql-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Using Freshservice On-Call Management</t>
+          <t>PostgreSQL Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003776-using-freshservice-on-call-management</t>
+          <t>https://help.savantlabs.io/en/articles/6565208-postgresql-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Configuring phone numbers correctly</t>
+          <t>Airtable Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009364-configuring-phone-numbers-correctly</t>
+          <t>https://help.savantlabs.io/en/articles/6666081-airtable-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Create an on-call schedule</t>
+          <t>Marketo Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009365-create-an-on-call-schedule</t>
+          <t>https://help.savantlabs.io/en/articles/6666851-marketo-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Creating an on-call shift</t>
+          <t>Databricks Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009366-creating-an-on-call-shift</t>
+          <t>https://help.savantlabs.io/en/articles/6739092-databricks-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Define and monitor services using Service Health Monitoring</t>
+          <t>Tableau Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004945-define-and-monitor-services-using-service-health-monitoring</t>
+          <t>https://help.savantlabs.io/en/articles/6801919-tableau-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Setting up Service Health Monitoring</t>
+          <t>Power BI Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006180-setting-up-service-health-monitoring</t>
+          <t>https://help.savantlabs.io/en/articles/6809525-power-bi-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Exploring Potential Services in Service Health Monitoring</t>
+          <t>SQL Server Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006181-exploring-potential-services-in-service-health-monitoring</t>
+          <t>https://help.savantlabs.io/en/articles/6946059-sql-server-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Deleting a service in Service Health Monitoring</t>
+          <t>December 2022 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006183-deleting-a-service-in-service-health-monitoring</t>
+          <t>https://help.savantlabs.io/en/articles/6978912-december-2022-updates</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Service Health Monitor for IT Asset Management</t>
+          <t>January 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000014260-service-health-monitor-for-it-asset-management</t>
+          <t>https://help.savantlabs.io/en/articles/6978924-january-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Working with major incidents in Freshservice</t>
+          <t>Facebook Ads Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006167-working-with-major-incidents-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/6980604-facebook-ads-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Preparing to work on a major incident</t>
+          <t>Google Ads Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006323-preparing-to-work-on-a-major-incident</t>
+          <t>https://help.savantlabs.io/en/articles/6988751-google-ads-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Setting up the Status Page</t>
+          <t>February 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006247-setting-up-the-status-page</t>
+          <t>https://help.savantlabs.io/en/articles/7017261-february-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Setting up collaboration apps</t>
+          <t>Generic API Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006338-setting-up-collaboration-apps</t>
+          <t>https://help.savantlabs.io/en/articles/7030173-generic-api-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Managing a Major Incident</t>
+          <t>Functions | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006363-managing-a-major-incident</t>
+          <t>https://help.savantlabs.io/en/articles/7048857-functions</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Setting up a Status Page</t>
+          <t>Google BigQuery Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009311-setting-up-a-status-page</t>
+          <t>https://help.savantlabs.io/en/articles/7097388-google-bigquery-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Customizing your Status Page</t>
+          <t>March 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009346-customizing-your-status-page</t>
+          <t>https://help.savantlabs.io/en/articles/7104711-march-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Managing subscribers of your Status Page</t>
+          <t>Baby Names Analytics: Exercise #1 | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009347-managing-subscribers-of-your-status-page</t>
+          <t>https://help.savantlabs.io/en/articles/7104716-baby-names-analytics-exercise-1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Fine tuning the security settings of the status page</t>
+          <t>Baby Names Analytics: Exercise #2 | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009912-fine-tuning-the-security-settings-of-the-status-page</t>
+          <t>https://help.savantlabs.io/en/articles/7104718-baby-names-analytics-exercise-2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Deleting the Status Page</t>
+          <t>Baby Names Analytics: Exercise #3 | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009348-deleting-the-status-page</t>
+          <t>https://help.savantlabs.io/en/articles/7104723-baby-names-analytics-exercise-3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Different Types of Assets/Configuration Items in Freshservice</t>
+          <t>Custom SSO Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/164410-different-types-of-assets-configuration-items-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/7118955-custom-sso-setup</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Adding Depreciation to assets in Freshservice</t>
+          <t>Google Analytics 4 Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/196934-adding-depreciation-to-assets-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/7183605-google-analytics-4-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Add new assets or configuration items manually</t>
+          <t>JIRA Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/164412-add-new-assets-or-configuration-items-manually</t>
+          <t>https://help.savantlabs.io/en/articles/7184858-jira-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Importing Assets</t>
+          <t>Microsoft Exchange Connector | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/234757-importing-assets</t>
+          <t>https://help.savantlabs.io/en/articles/7203648-microsoft-exchange-connector</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Viewing Information About Configurations Items in Freshservice</t>
+          <t>Microsoft Excel 365 Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/164413-viewing-information-about-configurations-items-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/7203983-microsoft-excel-365-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Basic Discovery tools and Cloud Discovery for IT asset management</t>
+          <t>Oracle DB Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/223633-basic-discovery-tools-and-cloud-discovery-for-it-asset-management</t>
+          <t>https://help.savantlabs.io/en/articles/7211531-oracle-db-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Freshservice Discovery Probe</t>
+          <t>Stripe Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/158679-freshservice-discovery-probe</t>
+          <t>https://help.savantlabs.io/en/articles/7211781-stripe-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IT asset attributes discovered by Discovery Agent and Probe</t>
+          <t>April 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/226174-it-asset-attributes-discovered-by-discovery-agent-and-probe</t>
+          <t>https://help.savantlabs.io/en/articles/7438086-april-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Managing IT assets with Discovery Hub</t>
+          <t>Opportunity Pipeline Change Report | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000010238-managing-it-assets-with-discovery-hub</t>
+          <t>https://help.savantlabs.io/en/articles/7879712-opportunity-pipeline-change-report</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Installing Discovery Agent [Windows]</t>
+          <t>SDR Productivity Kit: Meetings Preprocess | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/223635-installing-discovery-agent-windows-</t>
+          <t>https://help.savantlabs.io/en/articles/7934416-sdr-productivity-kit-meetings-preprocess</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Installing Discovery Agent [Win] in a Domain [using GPO]</t>
+          <t>Asset and Liability Reconciliation | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/199849-installing-discovery-agent-win-in-a-domain-using-gpo-</t>
+          <t>https://help.savantlabs.io/en/articles/7937058-asset-and-liability-reconciliation</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Freshservice Discovery Agent</t>
+          <t>Sales and Use Tax (Current Year) | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/200393-freshservice-discovery-agent</t>
+          <t>https://help.savantlabs.io/en/articles/7937143-sales-and-use-tax-current-year</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Installing Discovery Agent [Win] in a Workgroup [using PsExec]</t>
+          <t>SDR Productivity Kit: Outbound Touches Preprocess | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/199805-installing-discovery-agent-win-in-a-workgroup-using-psexec-</t>
+          <t>https://help.savantlabs.io/en/articles/7939082-sdr-productivity-kit-outbound-touches-preprocess</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Installing Discovery Agent [Mac]</t>
+          <t>SDR Productivity Kit: SDR Activity | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/205508-installing-discovery-agent-mac-</t>
+          <t>https://help.savantlabs.io/en/articles/7943470-sdr-productivity-kit-sdr-activity</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Downloading and installing the Discovery Probe</t>
+          <t>Download US Census Data into a Database | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/158680-downloading-and-installing-the-discovery-probe</t>
+          <t>https://help.savantlabs.io/en/articles/7943691-download-us-census-data-into-a-database</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>How to integrate SCCM with your Freshservice account</t>
+          <t>Adapter Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/205230-how-to-integrate-sccm-with-your-freshservice-account</t>
+          <t>https://help.savantlabs.io/en/articles/7943792-adapter-agent</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Configuring the Discovery Probe</t>
+          <t>Lead Funnel Metrics Report | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/158681-configuring-the-discovery-probe</t>
+          <t>https://help.savantlabs.io/en/articles/7946422-lead-funnel-metrics-report</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SNMP Device Discovery</t>
+          <t>Match Leads to Accounts | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/221269-snmp-device-discovery-</t>
+          <t>https://help.savantlabs.io/en/articles/7946546-match-leads-to-accounts</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Managing scanned assets and scan errors</t>
+          <t>Update Database from Spreadsheet Input with Email Alert | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/158682-managing-scanned-assets-and-scan-errors</t>
+          <t>https://help.savantlabs.io/en/articles/7947227-update-database-from-spreadsheet-input-with-email-alert</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Freshservice Cloud Discovery - Azure Cloud</t>
+          <t>Web Activity Analytics | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003721-freshservice-cloud-discovery-azure-cloud</t>
+          <t>https://help.savantlabs.io/en/articles/7947680-web-activity-analytics</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Freshservice Cloud Management - AWS Integration</t>
+          <t>How to Create Your Analysis | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003723-freshservice-cloud-management-aws-integration</t>
+          <t>https://help.savantlabs.io/en/articles/7968213-how-to-create-your-analysis</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Freshservice Cloud Discovery - VMware Vcenter</t>
+          <t>Connecting Data | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003772-freshservice-cloud-discovery-vmware-vcenter</t>
+          <t>https://help.savantlabs.io/en/articles/7970970-connecting-data</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Introduction to Freshservice Cloud Management</t>
+          <t>May 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004732-introduction-to-freshservice-cloud-management</t>
+          <t>https://help.savantlabs.io/en/articles/7974618-may-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Get started with Freshservice Cloud Management</t>
+          <t>The Tool Menu | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004733-get-started-with-freshservice-cloud-management</t>
+          <t>https://help.savantlabs.io/en/articles/8001513-the-tool-menu</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Adding Relationships to Your Assets</t>
+          <t>Publishing Data | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/164417-adding-relationships-to-your-assets</t>
+          <t>https://help.savantlabs.io/en/articles/8001531-publishing-data</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>What are the different types of relationships in Freshservice?</t>
+          <t>Adding a Template to Your Workspace | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002810-what-are-the-different-types-of-relationships-in-freshservice-</t>
+          <t>https://help.savantlabs.io/en/articles/8002579-adding-a-template-to-your-workspace</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Visualize relationships with asset relationship maps</t>
+          <t>The Canvas | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003704-visualize-relationships-with-asset-relationship-maps</t>
+          <t>https://help.savantlabs.io/en/articles/8002884-the-canvas</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Managing Software using Software Asset Management</t>
+          <t>Adding Tools to Your Analysis | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/232738-managing-software-using-software-asset-management</t>
+          <t>https://help.savantlabs.io/en/articles/8003136-adding-tools-to-your-analysis</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Software License Management</t>
+          <t>Tool Configuration | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/227986-software-license-management</t>
+          <t>https://help.savantlabs.io/en/articles/8007739-tool-configuration</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Stay on top of Software and SaaS usage with the Analytics Module</t>
+          <t>Renaming and Annotating Tools | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004105-stay-on-top-of-software-and-saas-usage-with-the-analytics-module</t>
+          <t>https://help.savantlabs.io/en/articles/8007780-renaming-and-annotating-tools</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>What is SaaS Management?</t>
+          <t>Deleting Tools and Connectors | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003270-what-is-saas-management-</t>
+          <t>https://help.savantlabs.io/en/articles/8007801-deleting-tools-and-connectors</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Discovering your SaaS Applications</t>
+          <t>Runs Overview | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003280-discovering-your-saas-applications</t>
+          <t>https://help.savantlabs.io/en/articles/8007838-runs-overview</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Classifying, Managing and Creating Licenses for your SaaS Applications</t>
+          <t>Enrich Leads with a Database | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003281-classifying-managing-and-creating-licenses-for-your-saas-applications</t>
+          <t>https://help.savantlabs.io/en/articles/8017347-enrich-leads-with-a-database</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Tracking insights for SaaS Applications</t>
+          <t>Rolling 30 Day Usage Report | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003282-tracking-insights-for-saas-applications</t>
+          <t>https://help.savantlabs.io/en/articles/8017430-rolling-30-day-usage-report</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Taking Insight-driven Actions on SaaS Applications</t>
+          <t>Market Penetration by US Geo | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003283-taking-insight-driven-actions-on-saas-applications</t>
+          <t>https://help.savantlabs.io/en/articles/8020936-market-penetration-by-us-geo</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Contract Management Setup Guide</t>
+          <t>Update Database with Spreadsheet Input | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/204473-contract-management-setup-guide</t>
+          <t>https://help.savantlabs.io/en/articles/8021054-update-database-with-spreadsheet-input</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Software License Types</t>
+          <t>Send Report from Database | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/227988-software-license-types</t>
+          <t>https://help.savantlabs.io/en/articles/8021451-send-report-from-database</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Software License Contracts</t>
+          <t>Schedules | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000001744-software-license-contracts</t>
+          <t>https://help.savantlabs.io/en/articles/8032714-schedules</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Overview of curated contract reports in Freshservice</t>
+          <t>June 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003654-overview-of-curated-contract-reports-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8105301-june-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Getting Started with Purchase Orders</t>
+          <t>Connecting Tools Together | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002755-getting-started-with-purchase-orders</t>
+          <t>https://help.savantlabs.io/en/articles/8125318-connecting-tools-together</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Creating a Purchase Order</t>
+          <t>Transform Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002756-creating-a-purchase-order</t>
+          <t>https://help.savantlabs.io/en/articles/8168220-transform-agent</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Managing Approvals for Purchase Orders</t>
+          <t>Unpivot Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002757-managing-approvals-for-purchase-orders</t>
+          <t>https://help.savantlabs.io/en/articles/8173466-unpivot-agent</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Adding Associations and Attachments</t>
+          <t>Pivot Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002758-adding-associations-and-attachments</t>
+          <t>https://help.savantlabs.io/en/articles/8174094-pivot-agent</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Receiving Items in a Purchase Order</t>
+          <t>Split Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003090-receiving-items-in-a-purchase-order</t>
+          <t>https://help.savantlabs.io/en/articles/8174198-split-agent</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Restricting trusted IPs</t>
+          <t>Stack Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/191587-restricting-trusted-ips</t>
+          <t>https://help.savantlabs.io/en/articles/8174584-stack-agent</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Restricting service desk access to certain domains</t>
+          <t>Sample Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/227155-restricting-service-desk-access-to-certain-domains</t>
+          <t>https://help.savantlabs.io/en/articles/8179000-sample-agent</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>EUC data centre migration: Here's what you should do</t>
+          <t>July 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/234149-euc-data-centre-migration-here-s-what-you-should-do-</t>
+          <t>https://help.savantlabs.io/en/articles/8180037-july-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Accessing Freshservice with Freshworks Account</t>
+          <t>Summarize Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/235010-accessing-freshservice-with-freshworks-account</t>
+          <t>https://help.savantlabs.io/en/articles/8182173-summarize-agent</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>​Access Freshservice With Freshworks Organization Account</t>
+          <t>Filter Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000001168--access-freshservice-with-freshworks-organization-account</t>
+          <t>https://help.savantlabs.io/en/articles/8202204-filter-agent</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Freshservice to discontinue support of SSLv3, switch to TLS</t>
+          <t>JSON Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/207703-freshservice-to-discontinue-support-of-sslv3-switch-to-tls</t>
+          <t>https://help.savantlabs.io/en/articles/8202398-json-agent</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Enabling TLS 1.2 in Internet Explorer</t>
+          <t>User Roles and Permissions | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/223838-enabling-tls-1-2-in-internet-explorer</t>
+          <t>https://help.savantlabs.io/en/articles/8202461-user-roles-and-permissions</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TLS 1.1 Support Deprecation</t>
+          <t>Time Series Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000001633-tls-1-1-support-deprecation</t>
+          <t>https://help.savantlabs.io/en/articles/8207851-time-series-agent</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>TLS 1.2 Strong Cipher Suites Compatibility</t>
+          <t>Analyses Overview | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005518-tls-1-2-strong-cipher-suites-compatibility</t>
+          <t>https://help.savantlabs.io/en/articles/8207944-analyses-overview</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Necessary configuration changes to ensure uninterrupted portal access.</t>
+          <t>Data Overview | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000010457-necessary-configuration-changes-to-ensure-uninterrupted-portal-access-</t>
+          <t>https://help.savantlabs.io/en/articles/8215107-data-overview</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>GDPR and Freshservice</t>
+          <t>Admin Overview | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/233145-gdpr-and-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8218751-admin-overview</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Freshservice Cookies</t>
+          <t>Microsoft Project Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/238944-freshservice-cookies</t>
+          <t>https://help.savantlabs.io/en/articles/8218903-microsoft-project-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>EU Standard Contractual Clauses is added to the Freshworks Data Processing Addendum</t>
+          <t>Systems | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/235746-eu-standard-contractual-clauses-is-added-to-the-freshworks-data-processing-addendum-</t>
+          <t>https://help.savantlabs.io/en/articles/8230037-systems</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Freshworks commitment towards HIPAA Compliance</t>
+          <t>Adding Systems | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/238705-freshworks-commitment-towards-hipaa-compliance</t>
+          <t>https://help.savantlabs.io/en/articles/8230045-adding-systems</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Step-by-step guide to add SPF and DKIM email authentication in Freshservice/Freshservice for Business Teams</t>
+          <t>System Management | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003933-step-by-step-guide-to-add-spf-and-dkim-email-authentication-in-freshservice-freshservice-for-business</t>
+          <t>https://help.savantlabs.io/en/articles/8230096-system-management</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Configure DMARC for Freshservice</t>
+          <t>Creating Datasets | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003934-configure-dmarc-for-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8230465-creating-datasets</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Allowlist Freshworks domains and IPs for Freshservice/Freshservice for Business Teams mail server users (US)</t>
+          <t>Using Datasets in Analyses | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003961-allowlist-freshworks-domains-and-ips-for-freshservice-freshservice-for-business-teams-mail-server-use</t>
+          <t>https://help.savantlabs.io/en/articles/8230484-using-datasets-in-analyses</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Allowlist Freshworks domains and IPs for Freshservice mail server users (EU)</t>
+          <t>Managing Datasets | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003962-allowlist-freshworks-domains-and-ips-for-freshservice-mail-server-users-eu-</t>
+          <t>https://help.savantlabs.io/en/articles/8230487-managing-datasets</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Allowlist Freshworks domains and IPs for Freshservice/Freshservice for Business Teams mail server users (India)</t>
+          <t>API Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003963-allowlist-freshworks-domains-and-ips-for-freshservice-freshservice-for-business-teams-mail-server-use</t>
+          <t>https://help.savantlabs.io/en/articles/8232926-api-agent</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Freddy AI Insights | Freddy AI Trust: Frequently Asked Questions (FAQs)</t>
+          <t>Infer Agent ✨ | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000011337-freddy-ai-insights-freddy-ai-trust-frequently-asked-questions-faqs-</t>
+          <t>https://help.savantlabs.io/en/articles/8238614-infer-agent</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Navigation and Dashboard</t>
+          <t>Xero Connector Guide | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>https://support.freshdesk.com/support/solutions/articles/240171-navigation-and-dashboard</t>
+          <t>https://help.savantlabs.io/en/articles/8252733-xero-connector-guide</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Customising Ticket Forms</t>
+          <t>Workday Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>https://support.freshdesk.com/support/solutions/articles/240176-customising-ticket-forms</t>
+          <t>https://help.savantlabs.io/en/articles/8252759-workday-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Working with the Ticket List page</t>
+          <t>Automate Your Analytics | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>https://support.freshdesk.com/support/solutions/articles/240180-working-with-the-ticket-list-page</t>
+          <t>https://help.savantlabs.io/en/articles/8258224-automate-your-analytics</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Working with the Ticket Details page</t>
+          <t>What Is Savant? | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>https://support.freshdesk.com/support/solutions/articles/240181-working-with-the-ticket-details-page</t>
+          <t>https://help.savantlabs.io/en/articles/8264720-what-is-savant</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Understanding Email Notifications</t>
+          <t>How to Sign Up for Savant | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>https://support.freshdesk.com/support/solutions/articles/50000004189-understanding-email-notifications</t>
+          <t>https://help.savantlabs.io/en/articles/8264759-how-to-sign-up-for-savant</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>What to Do if None of Your Emails are Getting Converted into Tickets</t>
+          <t>Your First 30 Days with Savant | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>https://support.freshdesk.com/support/solutions/articles/50000004193-what-to-do-if-none-of-your-emails-are-getting-converted-into-tickets</t>
+          <t>https://help.savantlabs.io/en/articles/8264763-your-first-30-days-with-savant</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>What to Do if Specific Emails are Not Getting Converted into Tickets</t>
+          <t>How to Get Help | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>https://support.freshdesk.com/support/solutions/articles/50000004194-what-to-do-if-specific-emails-are-not-getting-converted-into-tickets</t>
+          <t>https://help.savantlabs.io/en/articles/8264768-how-to-get-help</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>How to Send an Email Notification to an Agent when a Ticket is Created</t>
+          <t>Connecting to Data Sources and Data Destinations | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>https://support.freshdesk.com/support/solutions/articles/50000004195-how-to-send-an-email-notification-to-an-agent-when-a-ticket-is-created</t>
+          <t>https://help.savantlabs.io/en/articles/8265331-connecting-to-data-sources-and-data-destinations</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>How to Skip New Ticket Notifications for Specific Scenarios</t>
+          <t>Your All-in-One Home for Analytics | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>https://support.freshdesk.com/support/solutions/articles/50000004196-how-to-skip-new-ticket-notifications-for-specific-scenarios</t>
+          <t>https://help.savantlabs.io/en/articles/8282882-your-all-in-one-home-for-analytics</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Freshservice integration with Slack</t>
+          <t>August 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/219701-freshservice-integration-with-slack</t>
+          <t>https://help.savantlabs.io/en/articles/8295540-august-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Freshservice integration with DocuSign</t>
+          <t>SFTP/FTP Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/219377-freshservice-integration-with-docusign</t>
+          <t>https://help.savantlabs.io/en/articles/8295960-sftp-ftp-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Freshservice Integration with Atlassian JIRA</t>
+          <t>Google Gmail Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/191806-freshservice-integration-with-atlassian-jira</t>
+          <t>https://help.savantlabs.io/en/articles/8295961-google-gmail-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Freshservice integration with Freshbooks</t>
+          <t>Google Search Ads 360 Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/190604-freshservice-integration-with-freshbooks</t>
+          <t>https://help.savantlabs.io/en/articles/8295964-google-search-ads-360-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Understanding Connector App Tasks in Freshservice</t>
+          <t>Quickbooks Online Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009590-understanding-connector-app-tasks-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8295967-quickbooks-online-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Connector Apps in Freshservice/Freshservice for Business Teams - Overview</t>
+          <t>Flight Analytics | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009609-connector-apps-in-freshservice-freshservice-for-business-teams-overview</t>
+          <t>https://help.savantlabs.io/en/articles/8302536-flight-analytics</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Freshservice Integration with ServiceNow Connector</t>
+          <t>Cashflow Forecasting | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009991-freshservice-integration-with-servicenow-connector</t>
+          <t>https://help.savantlabs.io/en/articles/8360931-cashflow-forecasting</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Freshservice integration with ServiceDesk Plus</t>
+          <t>Finance KPI Analysis | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009992-freshservice-integration-with-servicedesk-plus</t>
+          <t>https://help.savantlabs.io/en/articles/8361008-finance-kpi-analysis</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Freshservice integration with Smartsheet</t>
+          <t>International Currencies and Tax Calculations | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000010227-freshservice-integration-with-smartsheet</t>
+          <t>https://help.savantlabs.io/en/articles/8361027-international-currencies-and-tax-calculations</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>How to work with workflow automator</t>
+          <t>Sales Tax Variance | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/232139-how-to-work-with-workflow-automator</t>
+          <t>https://help.savantlabs.io/en/articles/8361031-sales-tax-variance</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Using Webhooks with the Workflow Automator</t>
+          <t>Recursion Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/157143-using-webhooks-with-the-workflow-automator</t>
+          <t>https://help.savantlabs.io/en/articles/8391773-recursion-agent</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Setting Hierarchical Approvals for Service Requests (using Workflow Automator)</t>
+          <t>September 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/211198-setting-hierarchical-approvals-for-service-requests-using-workflow-automator-</t>
+          <t>https://help.savantlabs.io/en/articles/8443976-september-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Manage Reopening of Resolved/Closed Tickets With Thank You Detector</t>
+          <t>Dedupe Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000000064-manage-reopening-of-resolved-closed-tickets-with-thank-you-detector</t>
+          <t>https://help.savantlabs.io/en/articles/8561199-dedupe-agent</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Auto-assigning Tickets to Agents in a Group (Round Robin)</t>
+          <t>November 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/157134-auto-assigning-tickets-to-agents-in-a-group-round-robin-</t>
+          <t>https://help.savantlabs.io/en/articles/8568538-november-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Creating Custom Objects</t>
+          <t>DATE | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003117-creating-custom-objects</t>
+          <t>https://help.savantlabs.io/en/articles/8709258-date</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Using Custom Objects in Workflows</t>
+          <t>DATE_ADD | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003118-using-custom-objects-in-workflows</t>
+          <t>https://help.savantlabs.io/en/articles/8709266-date_add</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Importing and Exporting Custom Objects</t>
+          <t>DATE_DIFF | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003039-importing-and-exporting-custom-objects</t>
+          <t>https://help.savantlabs.io/en/articles/8709278-date_diff</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Lookups to Custom Objects</t>
+          <t>DATETIME | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003817-lookups-to-custom-objects</t>
+          <t>https://help.savantlabs.io/en/articles/8709299-datetime</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Introducing Freshworks Organization</t>
+          <t>DAY | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002932-introducing-freshworks-organization</t>
+          <t>https://help.savantlabs.io/en/articles/8712542-day</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Migrating Freshservice SSO to Freshworks Organization</t>
+          <t>DAY_OF_WEEK | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003339-migrating-freshservice-sso-to-freshworks-organization</t>
+          <t>https://help.savantlabs.io/en/articles/8712602-day_of_week</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Setting up SSO Policies in Freshworks Organization</t>
+          <t>DAY_OF_YEAR | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003526-setting-up-sso-policies-in-freshworks-organization</t>
+          <t>https://help.savantlabs.io/en/articles/8712607-day_of_year</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Upgrading MSP Mode Accounts to Freshworks Organization</t>
+          <t>DAYS_IN_MONTH | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003564-upgrading-msp-mode-accounts-to-freshworks-organization</t>
+          <t>https://help.savantlabs.io/en/articles/8712616-days_in_month</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Upgrading Multi-Account Configurations to Freshworks Organization</t>
+          <t>DAYS_IN_YEAR | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003565-upgrading-multi-account-configurations-to-freshworks-organization</t>
+          <t>https://help.savantlabs.io/en/articles/8712627-days_in_year</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Getting Started with the Analytics Platform</t>
+          <t>HOUR | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002911-getting-started-with-the-analytics-platform</t>
+          <t>https://help.savantlabs.io/en/articles/8712674-hour</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Generate intuitive reports using Analytics Pro</t>
+          <t>INTERVAL (Date) | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/233557-generate-intuitive-reports-using-analytics-pro</t>
+          <t>https://help.savantlabs.io/en/articles/8712681-interval-date</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Get started with Analytics Basic</t>
+          <t>INTERVAL (DateTime) | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000001711-get-started-with-analytics-basic</t>
+          <t>https://help.savantlabs.io/en/articles/8712684-interval-datetime</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Analytics Widgets Glossary</t>
+          <t>MINUTE | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000001029-analytics-widgets-glossary</t>
+          <t>https://help.savantlabs.io/en/articles/8712690-minute</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Scheduled Data Export</t>
+          <t>MONTH | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/238958-scheduled-data-export</t>
+          <t>https://help.savantlabs.io/en/articles/8712694-month</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Understanding the Service Desk at a Glance Report</t>
+          <t>NOW | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/164826-understanding-the-service-desk-at-a-glance-report</t>
+          <t>https://help.savantlabs.io/en/articles/8712699-now</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Understanding the Helpdesk at a Glance Report</t>
+          <t>QUARTER | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/164828-understanding-the-helpdesk-at-a-glance-report</t>
+          <t>https://help.savantlabs.io/en/articles/8712703-quarter</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>The Enterprise Reporting Suite</t>
+          <t>SECOND | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/168280-the-enterprise-reporting-suite</t>
+          <t>https://help.savantlabs.io/en/articles/8712851-second</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Asset Reports</t>
+          <t>TIME_PERIOD | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/222304-asset-reports</t>
+          <t>https://help.savantlabs.io/en/articles/8712855-time_period</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Understanding the Service Desk Performance Analysis Report</t>
+          <t>TIME_PERIOD_OFFSET | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/164832-understanding-the-service-desk-performance-analysis-report</t>
+          <t>https://help.savantlabs.io/en/articles/8712892-time_period_offset</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Centralized Credential Store</t>
+          <t>TODAY | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003816-centralized-credential-store</t>
+          <t>https://help.savantlabs.io/en/articles/8713060-today</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Introducing upgraded APIs - Freshservice Support</t>
+          <t>WEEK/WEEK_OF_YEAR | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004220-introducing-upgraded-apis-freshservice-support</t>
+          <t>https://help.savantlabs.io/en/articles/8713063-week-week_of_year</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Deprecating v1 APIs for Freshservice</t>
+          <t>YEAR | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006003-deprecating-v1-apis-for-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8713065-year</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>How to View Freshservice Subscription Details</t>
+          <t>TO_BOOLEAN | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004846-how-to-view-freshservice-subscription-details</t>
+          <t>https://help.savantlabs.io/en/articles/8713067-to_boolean</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>How to Manage a Freshservice Subscription during Trial</t>
+          <t>TO_DATE | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004847-how-to-manage-a-freshservice-subscription-during-trial</t>
+          <t>https://help.savantlabs.io/en/articles/8713074-to_date</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>How to Activate a Freshservice Subscription</t>
+          <t>TO_DATETIME | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004848-how-to-activate-a-freshservice-subscription</t>
+          <t>https://help.savantlabs.io/en/articles/8713078-to_datetime</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>How to Upgrade an Active Freshservice Subscription</t>
+          <t>TO_INTEGER | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004849-how-to-upgrade-an-active-freshservice-subscription</t>
+          <t>https://help.savantlabs.io/en/articles/8713083-to_integer</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Downgrading an Active Freshservice Subscription</t>
+          <t>TO_NUMBER | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004850-downgrading-an-active-freshservice-subscription</t>
+          <t>https://help.savantlabs.io/en/articles/8718579-to_number</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>App Installation Types in Freshservice</t>
+          <t>TO_TEXT | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000011810-app-installation-types-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8718607-to_text</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Data Usage Analytics</t>
+          <t>ABS | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000014074-data-usage-analytics</t>
+          <t>https://help.savantlabs.io/en/articles/8718632-abs</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Freshservice Onboarding Flow</t>
+          <t>CEILING | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/228572-freshservice-onboarding-flow</t>
+          <t>https://help.savantlabs.io/en/articles/8718641-ceiling</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Multi-language support for Freshservice</t>
+          <t>FLOOR | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000010732-multi-language-support-for-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8718661-floor</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>List of Dynamic Placeholders</t>
+          <t>GREATEST | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/239543-list-of-dynamic-placeholders</t>
+          <t>https://help.savantlabs.io/en/articles/8718690-greatest</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Managing Agents in Freshservice</t>
+          <t>LEAST | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/204591-managing-agents-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8718807-least</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Freshservice System Requirements</t>
+          <t>LOG | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/212225-freshservice-system-requirements</t>
+          <t>https://help.savantlabs.io/en/articles/8718815-log</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Branding your service desk with your name and theme</t>
+          <t>MOD | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/156514-branding-your-service-desk-with-your-name-and-theme</t>
+          <t>https://help.savantlabs.io/en/articles/8718824-mod</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Logging in and accessing your service desk</t>
+          <t>POWER | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/157126-logging-in-and-accessing-your-service-desk</t>
+          <t>https://help.savantlabs.io/en/articles/8718831-power</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Using a Vanity Support URL and pointing the CNAME in Freshservice</t>
+          <t>RANDOM | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/156516-using-a-vanity-support-url-and-pointing-the-cname-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8718838-random</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Configuring a custom SSL certificate for your service desk portal</t>
+          <t>ROUND | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/193075-configuring-a-custom-ssl-certificate-for-your-service-desk-portal</t>
+          <t>https://help.savantlabs.io/en/articles/8718841-round</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Requesting Changes</t>
+          <t>ROUNDDOWN | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000001761-requesting-changes</t>
+          <t>https://help.savantlabs.io/en/articles/8718846-rounddown</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Getting started with FreshThemes</t>
+          <t>ROUNDUP | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003059-getting-started-with-freshthemes</t>
+          <t>https://help.savantlabs.io/en/articles/8718864-roundup</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Portal layout basics</t>
+          <t>COALESCE | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003064-portal-layout-basics</t>
+          <t>https://help.savantlabs.io/en/articles/8718875-coalesce</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>What is Handlebars JS?</t>
+          <t>FIRST_NOT_EMPTY | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003065-what-is-handlebars-js-</t>
+          <t>https://help.savantlabs.io/en/articles/8718879-first_not_empty</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Palettes and Hex Codes</t>
+          <t>IF | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003060-palettes-and-hex-codes</t>
+          <t>https://help.savantlabs.io/en/articles/8718884-if</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Partials and Placeholders</t>
+          <t>IFS | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003066-partials-and-placeholders</t>
+          <t>https://help.savantlabs.io/en/articles/8718888-ifs</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Understanding Full-time vs. Occasional agents</t>
+          <t>IS_EMPTY | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/154758-understanding-full-time-vs-occasional-agents</t>
+          <t>https://help.savantlabs.io/en/articles/8719001-is_empty</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Setting up a Password Policy in Freshservice</t>
+          <t>JSON_FIELD | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/218835-setting-up-a-password-policy-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8719014-json_field</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Adding Custom Fields for Users (Requesters &amp; Agents) in Freshservice</t>
+          <t>JSON_SET | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/210046-adding-custom-fields-for-users-requesters-agents-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8719019-json_set</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Managing Requesters in Freshservice</t>
+          <t>CONCAT | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/154762-managing-requesters-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8719024-concat</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Monitor requester activity from a single timeline</t>
+          <t>HASH | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000013974-monitor-requester-activity-from-a-single-timeline</t>
+          <t>https://help.savantlabs.io/en/articles/8719042-hash</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Setting Up Active Directory Single Sign On (SSO) for Remote Authentication</t>
+          <t>HTML_ESCAPE | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/169196-setting-up-active-directory-single-sign-on-sso-for-remote-authentication</t>
+          <t>https://help.savantlabs.io/en/articles/8719059-html_escape</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Setting up Microsoft Azure AD Single Sign-on in Freshservice</t>
+          <t>LENGTH | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/203501-setting-up-microsoft-azure-ad-single-sign-on-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8719088-length</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Configure Active Directory SSO With JSON Web Token</t>
+          <t>LEVENSHTEIN | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000001173-configure-active-directory-sso-with-json-web-token</t>
+          <t>https://help.savantlabs.io/en/articles/8719098-levenshtein</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Set up form fields for tickets, problems, changes, releases, and tasks</t>
+          <t>LOWER | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/156449-set-up-form-fields-for-tickets-problems-changes-releases-and-tasks</t>
+          <t>https://help.savantlabs.io/en/articles/8719269-lower</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Using Dependent Fields with Tickets, Problems, Changes and Releases</t>
+          <t>PROPER | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/193550-using-dependent-fields-with-tickets-problems-changes-and-releases</t>
+          <t>https://help.savantlabs.io/en/articles/8719275-proper</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Understanding different types of Ticket Fields and their importance in Freshservice</t>
+          <t>REGEX_EXTRACT | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/156450-understanding-different-types-of-ticket-fields-and-their-importance-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8719282-regex_extract</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Understanding Dependent Fields</t>
+          <t>REGEX_MATCH | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/156451-understanding-dependent-fields</t>
+          <t>https://help.savantlabs.io/en/articles/8719290-regex_match</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Customizing Service Desk Statuses</t>
+          <t>REGEX_REPLACE | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/156452-customizing-service-desk-statuses</t>
+          <t>https://help.savantlabs.io/en/articles/8719298-regex_replace</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>How to schedule and post announcements in Freshservice?</t>
+          <t>REGEX_SEARCH | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/215323-how-to-schedule-and-post-announcements-in-freshservice-</t>
+          <t>https://help.savantlabs.io/en/articles/8719305-regex_search</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>How to access notifications in Freshservice</t>
+          <t>REPLACE | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/230351-how-to-access-notifications-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8723471-replace</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>How Search Works in Freshservice</t>
+          <t>REVERSE | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/231703-how-search-works-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8723482-reverse</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Configuring Email Notifications For New Tickets</t>
+          <t>SEARCH | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/156453-configuring-email-notifications-for-new-tickets</t>
+          <t>https://help.savantlabs.io/en/articles/8724784-search</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Managing Notifications for Problems, Changes and Releases</t>
+          <t>SOUNDEX | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/156454-managing-notifications-for-problems-changes-and-releases</t>
+          <t>https://help.savantlabs.io/en/articles/8724793-soundex</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Email Notification for Expiring Assets</t>
+          <t>SPLIT_PART | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/191017-email-notification-for-expiring-assets</t>
+          <t>https://help.savantlabs.io/en/articles/8724797-split_part</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Setting Email Notification for IP Restriction and addition/deletion of Agents</t>
+          <t>UNESCAPE_HTML | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/207238-setting-email-notification-for-ip-restriction-and-addition-deletion-of-agents</t>
+          <t>https://help.savantlabs.io/en/articles/8728613-unescape_html</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Configuring Multilingual Email Notifications</t>
+          <t>UPPER | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/225682-configuring-multilingual-email-notifications</t>
+          <t>https://help.savantlabs.io/en/articles/8728627-upper</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Migrating from SendGrid to Freshworks Email Service (US)</t>
+          <t>IN | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002688-migrating-from-sendgrid-to-freshworks-email-service-us-</t>
+          <t>https://help.savantlabs.io/en/articles/8732468-in</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Migrating from SendGrid to Freshworks Email Service (EU)</t>
+          <t>CASE ... WHEN ... | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002689-migrating-from-sendgrid-to-freshworks-email-service-eu-</t>
+          <t>https://help.savantlabs.io/en/articles/8732470-case-when</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Migrating from SendGrid to Freshworks Email Service (AU)</t>
+          <t>January 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002690-migrating-from-sendgrid-to-freshworks-email-service-au-</t>
+          <t>https://help.savantlabs.io/en/articles/8780469-january-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Migrating from SendGrid to Freshworks Email Service (IND)</t>
+          <t>Microsoft OneDrive Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002691-migrating-from-sendgrid-to-freshworks-email-service-ind-</t>
+          <t>https://help.savantlabs.io/en/articles/8862661-microsoft-onedrive-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>OS and Browser requirements to support custom domains in Freshservice</t>
+          <t>Adobe Analytics Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003761-os-and-browser-requirements-to-support-custom-domains-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/8872399-adobe-analytics-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Deprecation of Password-Based Authentication for Google &amp; Microsoft Email</t>
+          <t>Box Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004192-deprecation-of-password-based-authentication-for-google-microsoft-email</t>
+          <t>https://help.savantlabs.io/en/articles/8887379-box-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Freshservice List of Migration Items - May 2022</t>
+          <t>February 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004250-freshservice-list-of-migration-items-may-2022</t>
+          <t>https://help.savantlabs.io/en/articles/8931999-february-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Freshservice List of Migration Items - November 2022</t>
+          <t>December 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005520-freshservice-list-of-migration-items-november-2022</t>
+          <t>https://help.savantlabs.io/en/articles/8932200-december-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Freshservice Changes, Upgrades and Deprecations - November 2023</t>
+          <t>October 2023 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006294-freshservice-changes-upgrades-and-deprecations-november-2023</t>
+          <t>https://help.savantlabs.io/en/articles/8932494-october-2023-updates</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Build portals on the fly the no-code way</t>
+          <t>March 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005515-build-portals-on-the-fly-the-no-code-way</t>
+          <t>https://help.savantlabs.io/en/articles/9048833-march-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Common actions supported by No code portal builder</t>
+          <t>dbt Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005535-common-actions-supported-by-no-code-portal-builder</t>
+          <t>https://help.savantlabs.io/en/articles/9074580-dbt-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Managing Header and Banner sections</t>
+          <t>April 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005536-managing-header-and-banner-sections</t>
+          <t>https://help.savantlabs.io/en/articles/9190017-april-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Creating custom sections using widgets</t>
+          <t>X Ads (Twitter) Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005539-creating-custom-sections-using-widgets</t>
+          <t>https://help.savantlabs.io/en/articles/9298547-x-ads-twitter-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Customizing existing home page sections  - cards and tickets sections</t>
+          <t>May 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005540-customizing-existing-home-page-sections-cards-and-tickets-sections</t>
+          <t>https://help.savantlabs.io/en/articles/9319942-may-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Dark Mode</t>
+          <t>June 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009419-dark-mode</t>
+          <t>https://help.savantlabs.io/en/articles/9508445-june-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Migration Process via Public APIs for Freshservice Data Migration Partners</t>
+          <t>Format Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000010695-migration-process-via-public-apis-for-freshservice-data-migration-partners</t>
+          <t>https://help.savantlabs.io/en/articles/9509980-format-agent</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>How to migrate into Freshservice via Bulk APIs? [For Freshservice Data Migration Partners]</t>
+          <t>AWS FSx Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000011768-how-to-migrate-into-freshservice-via-bulk-apis-for-freshservice-data-migration-partners-</t>
+          <t>https://help.savantlabs.io/en/articles/9541129-aws-fsx-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>How to create and assign approvals in Freshservice?</t>
+          <t>IP Whitelisting Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000011144-how-to-create-and-assign-approvals-in-freshservice-</t>
+          <t>https://help.savantlabs.io/en/articles/9578820-ip-whitelisting-setup</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Important points to note for approval groups</t>
+          <t>July 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000011150-important-points-to-note-for-approval-groups</t>
+          <t>https://help.savantlabs.io/en/articles/9596956-july-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Get help with Employee Onboarding - Freshservice Support</t>
+          <t>REPEAT() | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/239003-get-help-with-employee-onboarding-freshservice-support</t>
+          <t>https://help.savantlabs.io/en/articles/9650328-repeat</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Bulk Employee Onboarding in Freshservice</t>
+          <t>Microsoft Sharepoint Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/239640-bulk-employee-onboarding-in-freshservice</t>
+          <t>https://help.savantlabs.io/en/articles/9682338-microsoft-sharepoint-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Adding Stakeholders to the Onboarding Module</t>
+          <t>X Search (Twitter) Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002363-adding-stakeholders-to-the-onboarding-module</t>
+          <t>https://help.savantlabs.io/en/articles/9682647-x-search-twitter-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Building Onboarding Kits</t>
+          <t>NetSuite Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002364-building-onboarding-kits</t>
+          <t>https://help.savantlabs.io/en/articles/9715906-netsuite-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Creating Onboarding Tickets</t>
+          <t>Azure Synapse Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000002365-creating-onboarding-tickets</t>
+          <t>https://help.savantlabs.io/en/articles/9731251-azure-synapse-setup</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>What is a workspace?</t>
+          <t>Adding Users to Workspaces | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005551-what-is-a-workspace-</t>
+          <t>https://help.savantlabs.io/en/articles/9757487-adding-users-to-workspaces</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>What is a primary workspace?</t>
+          <t>August 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005552-what-is-a-primary-workspace-</t>
+          <t>https://help.savantlabs.io/en/articles/9829198-august-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>What is a ticket type or prefix?</t>
+          <t>Network Share Drive Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005527-what-is-a-ticket-type-or-prefix-</t>
+          <t>https://help.savantlabs.io/en/articles/9830936-network-share-drive-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Workspace Views</t>
+          <t>September 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005586-workspace-views</t>
+          <t>https://help.savantlabs.io/en/articles/9958964-september-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Moving data between workspaces: guidelines and restrictions</t>
+          <t>Contact Us | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005587-moving-data-between-workspaces-guidelines-and-restrictions</t>
+          <t>https://help.savantlabs.io/en/articles/9967033-contact-us</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Document generation for employee requests</t>
+          <t>Blend Agent | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000006197-document-generation-for-employee-requests</t>
+          <t>https://help.savantlabs.io/en/articles/9971999-blend-agent</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Embed eSignatures in Documents</t>
+          <t>Removing Users from Workspaces | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000009752-embed-esignatures-in-documents</t>
+          <t>https://help.savantlabs.io/en/articles/9972030-removing-users-from-workspaces</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Manage documents with the centralized list view</t>
+          <t>Importing a Savant Analysis | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000012015-manage-documents-with-the-centralized-list-view</t>
+          <t>https://help.savantlabs.io/en/articles/9981091-importing-a-savant-analysis</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Docusign for e-signatures in documents</t>
+          <t>October 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000011505-docusign-for-e-signatures-in-documents</t>
+          <t>https://help.savantlabs.io/en/articles/9999411-october-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Get started with project management</t>
+          <t>Smartsheet Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003092-get-started-with-project-management</t>
+          <t>https://help.savantlabs.io/en/articles/10011008-smartsheet-connector-setup</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Getting started with Contextual Collaboration in Projects via Slack</t>
+          <t>Triggers | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003605-getting-started-with-contextual-collaboration-in-projects-via-slack</t>
+          <t>https://help.savantlabs.io/en/articles/10064959-triggers</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Configuring high-level project automation settings from the admin</t>
+          <t>Re-authenticate a System | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003683-configuring-high-level-project-automation-settings-from-the-admin</t>
+          <t>https://help.savantlabs.io/en/articles/10067903-re-authenticate-a-system</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>How to configure your project settings?</t>
+          <t>PAD_LEFT | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003265-how-to-configure-your-project-settings-</t>
+          <t>https://help.savantlabs.io/en/articles/10202686-pad_left</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Projects not loading? Here is how to fix the problem</t>
+          <t>PAD_RIGHT | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000003047-projects-not-loading-here-is-how-to-fix-the-problem</t>
+          <t>https://help.savantlabs.io/en/articles/10203157-pad_right</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Introduction to Workload Management</t>
+          <t>LEFT_PART | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004723-introduction-to-workload-management</t>
+          <t>https://help.savantlabs.io/en/articles/10203195-left_part</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>How is workload calculated?</t>
+          <t>RIGHT_PART | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004752-how-is-workload-calculated-</t>
+          <t>https://help.savantlabs.io/en/articles/10203214-right_part</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>How can you visualize workload?</t>
+          <t>November 2024 Updates | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004756-how-can-you-visualize-workload-</t>
+          <t>https://help.savantlabs.io/en/articles/10207266-november-2024-updates</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Managing assigned and unassigned work via the workload module</t>
+          <t>CONTAINS | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000004757-managing-assigned-and-unassigned-work-via-the-workload-module</t>
+          <t>https://help.savantlabs.io/en/articles/10222841-contains</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Work Calendar</t>
+          <t>Klaviyo Connector Setup | Savant Labs, Inc. Help Center</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>https://support.freshservice.com/support/solutions/articles/50000005622-work-calendar</t>
+          <t>https://help.savantlabs.io/en/articles/10244994-klaviyo-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>MID | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10245054-mid</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>AVG | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10247408-avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>CONCAT | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250725-concat</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>CONCAT DISTINCT | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250740-concat-distinct</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>COUNT | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250749-count</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>COUNT DISTINCT | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250760-count-distinct</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>CUMULATIVE SUM | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250797-cumulative-sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>FILL | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250804-fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>FIRST | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250816-first</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>LAG | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250827-lag</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>LAST | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250829-last</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>LEAD | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250837-lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>MAX | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250840-max</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>MEDIAN | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250846-median</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>MIN | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250871-min</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>NTILE | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250994-ntile</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>RANK | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10250999-rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>ROW NUMBER | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10251003-row-number</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>STDDEV | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10251009-stddev</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>SUM | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10251013-sum</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>VAR | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10251017-var</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Run History | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10270513-run-history</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Flat File Datasets | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10279829-flat-file-datasets</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Audit Run Changes | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10291995-audit-run-changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>December 2024 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10309607-december-2024-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>January 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10486733-january-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>JWT_ENCODE | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10517511-jwt_encode</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>February 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10731243-february-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Explode Agent | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10732209-explode-agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>March 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/10861298-march-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Oracle Fusion Cloud Financials Connector Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11066100-oracle-fusion-cloud-financials-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>XML Agent | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11170724-xml-agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Notes Agent | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11172618-notes-agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Microsoft OneDrive/Sharepoint Connector | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11383444-microsoft-onedrive-sharepoint-connector</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>April 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11431908-april-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>May 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11432133-may-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>How OAuth Authentication works in Savant | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11462281-how-oauth-authentication-works-in-savant</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>OpenAI Connector Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11463773-openai-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>ADP Connector Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11557030-adp-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>TRIM | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11586103-trim</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>June 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11670067-june-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Sprinklr Connector Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11692808-sprinklr-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>July 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11898824-july-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>GEO_DISTANCE | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11909862-geo_distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Geocoding | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11914633-geocoding</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Distance &amp; Drive Time Analytics | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11914651-distance-drive-time-analytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Proximity Joins &amp; Service Areas | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11914670-proximity-joins-service-areas</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Nearest Neighbor &amp; Clustering | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/11914680-nearest-neighbor-clustering</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>August 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12043257-august-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>AI Agent for Messy Files | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12068343-ai-agent-for-messy-files</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>SAP HANA Database Connector Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12110205-sap-hana-database-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Microsoft Fabric Warehouse Connector Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12132607-microsoft-fabric-warehouse-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Automating Hierarchies: Iterative Logic Meets the Recursion Tool | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12142624-automating-hierarchies-iterative-logic-meets-the-recursion-tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>September 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12167020-september-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>AI Categorization &amp; Smart Tagging Agent | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12220150-ai-categorization-smart-tagging-agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Azure APIM Authentication Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12498487-azure-apim-authentication-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Anaplan Connector Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12541031-anaplan-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>October 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12573680-october-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>November 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12745509-november-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>LIST_TO_TEXT | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12805365-list_to_text</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Theobald Xtract Universal for SAP Connector Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/12986835-theobald-xtract-universal-for-sap-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>December 2025 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/13014599-december-2025-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Advanced Audit &amp; Activity Logs | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/13217686-advanced-audit-activity-logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Google Gemini Connector Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/13440871-google-gemini-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>How Slack OAuth Authentication works in Savant | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/13488962-how-slack-oauth-authentication-works-in-savant</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>January 2026 Updates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/13600951-january-2026-updates</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Savant Logs Guide | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/13654453-savant-logs-guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Write to SAP S/4HANA using the API Tool | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/13853911-write-to-sap-s-4hana-using-the-api-tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Microsoft Fabric Lakehouse Connector Setup | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/13972818-microsoft-fabric-lakehouse-connector-setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>February 2026 | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14006555-february-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Vision Agent ✨ | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14094408-vision-agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Fuse Agent ✨ | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14094437-fuse-agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Spatial Match Agent 🌎 | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14461037-spatial-match-agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Spatial Summarize Agent 🌎 | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14461320-spatial-summarize-agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>GEO_SPATIAL_DISTANCE | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14462645-geo_spatial_distance</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>GEO_POINT | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14462789-geo_point</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>GEO_TYPE | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14462975-geo_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>GEO_AREA | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14463085-geo_area</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>GEO_CENTROID | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14463134-geo_centroid</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>GEO_DIFFERENCE | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14464039-geo_difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>GEO_UNION | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14464058-geo_union</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>GEO_INTERSECTION | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14464084-geo_intersection</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>GEO_BUFFER | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14464101-geo_buffer</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>GEO_TRADE_AREA | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14464361-geo_trade_area</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>GEO_PERIMETER | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14464408-geo_perimeter</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>GEO_ISVALID | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14464460-geo_isvalid</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Files Overview | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14780016-files-overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Flat Files and Text Blobs | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14780483-flat-files-and-text-blobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Spreadsheets (Excel + Google Sheets) | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14780656-spreadsheets-excel-google-sheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>PDF | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14885454-pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Parquet | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14886167-parquet</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>How can I resolve column ordering issues in the Pivot Tool? | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14961446-how-can-i-resolve-column-ordering-issues-in-the-pivot-tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>How can I troubleshoot workflow analysis errors in Savant? | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/articles/14961608-how-can-i-troubleshoot-workflow-analysis-errors-in-savant</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>What's New | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/collections/3850665-what-s-new</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Getting Started | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/collections/4065910-getting-started</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Product Walkthrough | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/collections/3345890-product-walkthrough</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Agents and Functions | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/collections/4065822-agents-and-functions</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Connectors and Files | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/collections/3480481-connectors-and-files</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Templates | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/collections/3642171-templates</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Contact Us | Savant Labs, Inc. Help Center</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/collections/10591935-contact-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr"/>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>https://help.savantlabs.io/en/collections/3979532-tips-tricks</t>
         </is>
       </c>
     </row>

</xml_diff>